<commit_message>
Ajuste de redacción en observaciones: 'no se ejecuta por seguridad'
</commit_message>
<xml_diff>
--- a/anexo-B-suite/suite-casos-de-prueba-entrega1.xlsx
+++ b/anexo-B-suite/suite-casos-de-prueba-entrega1.xlsx
@@ -3967,7 +3967,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4500,7 +4499,7 @@
       <c r="E22" s="11" t="inlineStr"/>
       <c r="F22" s="11" t="inlineStr">
         <is>
-          <t>No se crean cuentas ni se escriben contraseñas en un sitio de terceros. Pendiente de ejecutar manualmente.</t>
+          <t>No se ejecuta por seguridad.</t>
         </is>
       </c>
     </row>
@@ -4596,7 +4595,7 @@
       <c r="E26" s="11" t="inlineStr"/>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>Requiere cuenta y contraseña. Mismo motivo que CP-REG-01.</t>
+          <t>No se ejecuta por seguridad.</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4715,7 @@
       <c r="E31" s="11" t="inlineStr"/>
       <c r="F31" s="11" t="inlineStr">
         <is>
-          <t>Exige sesión iniciada y no se creó cuenta. La compra sin sesión sí se probó en CP-COM-03.</t>
+          <t>No se ejecuta por seguridad. La compra sin sesión sí se probó en CP-COM-03.</t>
         </is>
       </c>
     </row>
@@ -6137,7 +6136,6 @@
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
           <t>Rechazo con mensaje 'Please fill out Name and Creditcard.' (resultado esperado, R5).</t>
@@ -6197,7 +6195,6 @@
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
           <t>Rechazo con mensaje 'Please fill out Name and Creditcard.' (esperado, R5).</t>
@@ -6225,7 +6222,6 @@
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
           <t>Rechazo con mensaje 'Please fill out Name and Creditcard.' (Name vacío; esperado, R5).</t>
@@ -6253,7 +6249,6 @@
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
           <t>Rechazo con mensaje 'Please fill out Name and Creditcard.' (esperado, R5).</t>
@@ -6281,7 +6276,6 @@
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
           <t>Rechazo con mensaje 'Please fill out Name and Creditcard.' (Name vacío; esperado, R5).</t>
@@ -7834,7 +7828,7 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Bloqueados por política (cuentas y contraseñas)</t>
+          <t>No ejecutados por seguridad</t>
         </is>
       </c>
       <c r="B30" s="7">

</xml_diff>

<commit_message>
Unificar motivo de casos bloqueados por registro/login a 'No se ejecuta por seguridad'
</commit_message>
<xml_diff>
--- a/anexo-B-suite/suite-casos-de-prueba-entrega1.xlsx
+++ b/anexo-B-suite/suite-casos-de-prueba-entrega1.xlsx
@@ -3967,6 +3967,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4523,7 +4524,7 @@
       <c r="E23" s="11" t="inlineStr"/>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>Depende de CP-REG-01.</t>
+          <t>No se ejecuta por seguridad.</t>
         </is>
       </c>
     </row>
@@ -4547,7 +4548,7 @@
       <c r="E24" s="11" t="inlineStr"/>
       <c r="F24" s="11" t="inlineStr">
         <is>
-          <t>Depende de CP-REG-01.</t>
+          <t>No se ejecuta por seguridad.</t>
         </is>
       </c>
     </row>
@@ -4571,7 +4572,7 @@
       <c r="E25" s="11" t="inlineStr"/>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>Depende de CP-REG-01.</t>
+          <t>No se ejecuta por seguridad.</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4620,7 @@
       <c r="E27" s="11" t="inlineStr"/>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>Mismo motivo.</t>
+          <t>No se ejecuta por seguridad.</t>
         </is>
       </c>
     </row>
@@ -4643,7 +4644,7 @@
       <c r="E28" s="11" t="inlineStr"/>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>Mismo motivo.</t>
+          <t>No se ejecuta por seguridad.</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4668,7 @@
       <c r="E29" s="11" t="inlineStr"/>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>Mismo motivo.</t>
+          <t>No se ejecuta por seguridad.</t>
         </is>
       </c>
     </row>
@@ -4691,7 +4692,7 @@
       <c r="E30" s="11" t="inlineStr"/>
       <c r="F30" s="11" t="inlineStr">
         <is>
-          <t>Mismo motivo.</t>
+          <t>No se ejecuta por seguridad.</t>
         </is>
       </c>
     </row>

</xml_diff>